<commit_message>
update [starfish] 种子词库_第二次输出_v3_含CMF专著.xlsx (195 words, CMF as normal corpus)
</commit_message>
<xml_diff>
--- a/种子词库_第二次输出_v3_含CMF专著.xlsx
+++ b/种子词库_第二次输出_v3_含CMF专著.xlsx
@@ -31,7 +31,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -41,11 +41,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -84,12 +79,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -457,18 +446,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I175"/>
+  <dimension ref="A1:G196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,16 +494,6 @@
           <t>语料频次</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>是否CMF专著新增</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -554,8 +531,6 @@
       <c r="G2" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr"/>
@@ -579,8 +554,6 @@
       <c r="G3" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr"/>
@@ -606,8 +579,6 @@
       <c r="G4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr"/>
@@ -633,8 +604,6 @@
       <c r="G5" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr"/>
@@ -660,8 +629,6 @@
       <c r="G6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr"/>
@@ -686,8 +653,6 @@
       <c r="G7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr"/>
@@ -715,8 +680,6 @@
       <c r="G8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr"/>
@@ -740,8 +703,6 @@
       <c r="G9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr"/>
@@ -771,8 +732,6 @@
       <c r="G10" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr"/>
@@ -798,8 +757,6 @@
       <c r="G11" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr"/>
@@ -833,8 +790,6 @@
       <c r="G12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr"/>
@@ -862,8 +817,6 @@
       <c r="G13" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr"/>
@@ -893,8 +846,6 @@
       <c r="G14" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr"/>
@@ -920,8 +871,6 @@
       <c r="G15" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -957,8 +906,6 @@
       <c r="G16" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr"/>
@@ -982,8 +929,6 @@
       <c r="G17" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr"/>
@@ -1007,8 +952,6 @@
       <c r="G18" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr"/>
@@ -1032,8 +975,6 @@
       <c r="G19" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr"/>
@@ -1057,8 +998,6 @@
       <c r="G20" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr"/>
@@ -1082,8 +1021,6 @@
       <c r="G21" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr"/>
@@ -1110,8 +1047,6 @@
       <c r="G22" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr"/>
@@ -1135,8 +1070,6 @@
       <c r="G23" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr"/>
@@ -1164,8 +1097,6 @@
       <c r="G24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr"/>
@@ -1189,8 +1120,6 @@
       <c r="G25" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr"/>
@@ -1214,8 +1143,6 @@
       <c r="G26" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr"/>
@@ -1239,8 +1166,6 @@
       <c r="G27" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr"/>
@@ -1276,8 +1201,6 @@
       <c r="G28" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr"/>
@@ -1301,8 +1224,6 @@
       <c r="G29" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr"/>
@@ -1326,8 +1247,6 @@
       <c r="G30" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr"/>
@@ -1351,8 +1270,6 @@
       <c r="G31" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr"/>
@@ -1380,8 +1297,6 @@
       <c r="G32" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr"/>
@@ -1405,8 +1320,6 @@
       <c r="G33" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr"/>
@@ -1430,8 +1343,6 @@
       <c r="G34" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr"/>
@@ -1455,8 +1366,6 @@
       <c r="G35" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr"/>
@@ -1480,8 +1389,6 @@
       <c r="G36" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr"/>
@@ -1505,8 +1412,6 @@
       <c r="G37" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr"/>
@@ -1538,8 +1443,6 @@
       <c r="G38" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr"/>
@@ -1563,8 +1466,6 @@
       <c r="G39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr"/>
@@ -1588,8 +1489,6 @@
       <c r="G40" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr"/>
@@ -1613,8 +1512,6 @@
       <c r="G41" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr"/>
@@ -1638,8 +1535,6 @@
       <c r="G42" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr"/>
@@ -1663,8 +1558,6 @@
       <c r="G43" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr"/>
@@ -1688,8 +1581,6 @@
       <c r="G44" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr"/>
@@ -1713,8 +1604,6 @@
       <c r="G45" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H45" s="2" t="inlineStr"/>
-      <c r="I45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr"/>
@@ -1742,8 +1631,6 @@
       <c r="G46" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr"/>
@@ -1767,8 +1654,6 @@
       <c r="G47" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr"/>
@@ -1792,8 +1677,6 @@
       <c r="G48" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr"/>
@@ -1817,8 +1700,6 @@
       <c r="G49" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H49" s="2" t="inlineStr"/>
-      <c r="I49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr"/>
@@ -1845,8 +1726,6 @@
       <c r="G50" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr"/>
@@ -1873,8 +1752,6 @@
       <c r="G51" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H51" s="2" t="inlineStr"/>
-      <c r="I51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr"/>
@@ -1902,8 +1779,6 @@
       <c r="G52" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr"/>
@@ -1927,8 +1802,6 @@
       <c r="G53" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H53" s="2" t="inlineStr"/>
-      <c r="I53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr"/>
@@ -1952,8 +1825,6 @@
       <c r="G54" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr"/>
@@ -1977,8 +1848,6 @@
       <c r="G55" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H55" s="2" t="inlineStr"/>
-      <c r="I55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr"/>
@@ -2002,8 +1871,6 @@
       <c r="G56" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr"/>
@@ -2035,8 +1902,6 @@
       <c r="G57" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H57" s="2" t="inlineStr"/>
-      <c r="I57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr"/>
@@ -2060,8 +1925,6 @@
       <c r="G58" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H58" s="2" t="inlineStr"/>
-      <c r="I58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr"/>
@@ -2085,8 +1948,6 @@
       <c r="G59" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H59" s="2" t="inlineStr"/>
-      <c r="I59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr"/>
@@ -2110,8 +1971,6 @@
       <c r="G60" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr"/>
@@ -2135,8 +1994,6 @@
       <c r="G61" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H61" s="2" t="inlineStr"/>
-      <c r="I61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr"/>
@@ -2160,8 +2017,6 @@
       <c r="G62" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H62" s="2" t="inlineStr"/>
-      <c r="I62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr"/>
@@ -2192,8 +2047,6 @@
       <c r="G63" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H63" s="2" t="inlineStr"/>
-      <c r="I63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr"/>
@@ -2217,8 +2070,6 @@
       <c r="G64" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr"/>
@@ -2242,8 +2093,6 @@
       <c r="G65" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H65" s="2" t="inlineStr"/>
-      <c r="I65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr"/>
@@ -2267,8 +2116,6 @@
       <c r="G66" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H66" s="2" t="inlineStr"/>
-      <c r="I66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr"/>
@@ -2292,8 +2139,6 @@
       <c r="G67" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H67" s="2" t="inlineStr"/>
-      <c r="I67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr"/>
@@ -2317,8 +2162,6 @@
       <c r="G68" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H68" s="2" t="inlineStr"/>
-      <c r="I68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr"/>
@@ -2345,8 +2188,6 @@
       <c r="G69" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H69" s="2" t="inlineStr"/>
-      <c r="I69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr"/>
@@ -2378,8 +2219,6 @@
       <c r="G70" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr"/>
@@ -2403,8 +2242,6 @@
       <c r="G71" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H71" s="2" t="inlineStr"/>
-      <c r="I71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr"/>
@@ -2428,8 +2265,6 @@
       <c r="G72" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr"/>
@@ -2457,8 +2292,6 @@
       <c r="G73" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H73" s="2" t="inlineStr"/>
-      <c r="I73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr"/>
@@ -2482,8 +2315,6 @@
       <c r="G74" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr"/>
@@ -2509,8 +2340,6 @@
       <c r="G75" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H75" s="2" t="inlineStr"/>
-      <c r="I75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr"/>
@@ -2536,8 +2365,6 @@
       <c r="G76" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H76" s="2" t="inlineStr"/>
-      <c r="I76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr"/>
@@ -2561,8 +2388,6 @@
       <c r="G77" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H77" s="2" t="inlineStr"/>
-      <c r="I77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr"/>
@@ -2586,8 +2411,6 @@
       <c r="G78" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H78" s="2" t="inlineStr"/>
-      <c r="I78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr"/>
@@ -2611,8 +2434,6 @@
       <c r="G79" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H79" s="2" t="inlineStr"/>
-      <c r="I79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr"/>
@@ -2636,8 +2457,6 @@
       <c r="G80" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H80" s="2" t="inlineStr"/>
-      <c r="I80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr"/>
@@ -2665,8 +2484,6 @@
       <c r="G81" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H81" s="2" t="inlineStr"/>
-      <c r="I81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr"/>
@@ -2690,8 +2507,6 @@
       <c r="G82" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H82" s="2" t="inlineStr"/>
-      <c r="I82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr"/>
@@ -2715,8 +2530,6 @@
       <c r="G83" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H83" s="2" t="inlineStr"/>
-      <c r="I83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr"/>
@@ -2740,8 +2553,6 @@
       <c r="G84" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="H84" s="2" t="inlineStr"/>
-      <c r="I84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr"/>
@@ -2765,8 +2576,6 @@
       <c r="G85" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H85" s="2" t="inlineStr"/>
-      <c r="I85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr"/>
@@ -2790,8 +2599,6 @@
       <c r="G86" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H86" s="2" t="inlineStr"/>
-      <c r="I86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr"/>
@@ -2815,8 +2622,6 @@
       <c r="G87" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H87" s="2" t="inlineStr"/>
-      <c r="I87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2857,8 +2662,6 @@
       <c r="G88" s="2" t="n">
         <v>418</v>
       </c>
-      <c r="H88" s="2" t="inlineStr"/>
-      <c r="I88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr"/>
@@ -2886,8 +2689,6 @@
       <c r="G89" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="H89" s="2" t="inlineStr"/>
-      <c r="I89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr"/>
@@ -2916,8 +2717,6 @@
       <c r="G90" s="2" t="n">
         <v>253</v>
       </c>
-      <c r="H90" s="2" t="inlineStr"/>
-      <c r="I90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr"/>
@@ -2941,8 +2740,6 @@
       <c r="G91" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H91" s="2" t="inlineStr"/>
-      <c r="I91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr"/>
@@ -2968,8 +2765,6 @@
       <c r="G92" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H92" s="2" t="inlineStr"/>
-      <c r="I92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr"/>
@@ -2995,8 +2790,6 @@
       <c r="G93" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H93" s="2" t="inlineStr"/>
-      <c r="I93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr"/>
@@ -3020,8 +2813,6 @@
       <c r="G94" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H94" s="2" t="inlineStr"/>
-      <c r="I94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr"/>
@@ -3047,8 +2838,6 @@
       <c r="G95" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H95" s="2" t="inlineStr"/>
-      <c r="I95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr"/>
@@ -3072,8 +2861,6 @@
       <c r="G96" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H96" s="2" t="inlineStr"/>
-      <c r="I96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr"/>
@@ -3099,8 +2886,6 @@
       <c r="G97" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H97" s="2" t="inlineStr"/>
-      <c r="I97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr"/>
@@ -3127,8 +2912,6 @@
       <c r="G98" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H98" s="2" t="inlineStr"/>
-      <c r="I98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr"/>
@@ -3157,8 +2940,6 @@
       <c r="G99" s="2" t="n">
         <v>273</v>
       </c>
-      <c r="H99" s="2" t="inlineStr"/>
-      <c r="I99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr"/>
@@ -3186,8 +2967,6 @@
       <c r="G100" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H100" s="2" t="inlineStr"/>
-      <c r="I100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr"/>
@@ -3211,8 +2990,6 @@
       <c r="G101" s="2" t="n">
         <v>110</v>
       </c>
-      <c r="H101" s="2" t="inlineStr"/>
-      <c r="I101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr"/>
@@ -3236,8 +3013,6 @@
       <c r="G102" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H102" s="2" t="inlineStr"/>
-      <c r="I102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr"/>
@@ -3261,8 +3036,6 @@
       <c r="G103" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H103" s="2" t="inlineStr"/>
-      <c r="I103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr"/>
@@ -3286,8 +3059,6 @@
       <c r="G104" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H104" s="2" t="inlineStr"/>
-      <c r="I104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr"/>
@@ -3315,8 +3086,6 @@
       <c r="G105" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="H105" s="2" t="inlineStr"/>
-      <c r="I105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr"/>
@@ -3340,8 +3109,6 @@
       <c r="G106" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H106" s="2" t="inlineStr"/>
-      <c r="I106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr"/>
@@ -3365,8 +3132,6 @@
       <c r="G107" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H107" s="2" t="inlineStr"/>
-      <c r="I107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr"/>
@@ -3392,8 +3157,6 @@
       <c r="G108" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H108" s="2" t="inlineStr"/>
-      <c r="I108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr"/>
@@ -3417,8 +3180,6 @@
       <c r="G109" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H109" s="2" t="inlineStr"/>
-      <c r="I109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr"/>
@@ -3442,8 +3203,6 @@
       <c r="G110" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H110" s="2" t="inlineStr"/>
-      <c r="I110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr"/>
@@ -3478,8 +3237,6 @@
       <c r="G111" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="H111" s="2" t="inlineStr"/>
-      <c r="I111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr"/>
@@ -3503,8 +3260,6 @@
       <c r="G112" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="H112" s="2" t="inlineStr"/>
-      <c r="I112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr"/>
@@ -3530,8 +3285,6 @@
       <c r="G113" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="H113" s="2" t="inlineStr"/>
-      <c r="I113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr"/>
@@ -3557,8 +3310,6 @@
       <c r="G114" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="H114" s="2" t="inlineStr"/>
-      <c r="I114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr"/>
@@ -3585,8 +3336,6 @@
       <c r="G115" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H115" s="2" t="inlineStr"/>
-      <c r="I115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr"/>
@@ -3612,8 +3361,6 @@
       <c r="G116" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H116" s="2" t="inlineStr"/>
-      <c r="I116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr"/>
@@ -3639,8 +3386,6 @@
       <c r="G117" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H117" s="2" t="inlineStr"/>
-      <c r="I117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr"/>
@@ -3670,8 +3415,6 @@
       <c r="G118" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H118" s="2" t="inlineStr"/>
-      <c r="I118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr"/>
@@ -3700,8 +3443,6 @@
       <c r="G119" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H119" s="2" t="inlineStr"/>
-      <c r="I119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr"/>
@@ -3733,8 +3474,6 @@
       <c r="G120" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="H120" s="2" t="inlineStr"/>
-      <c r="I120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr"/>
@@ -3761,8 +3500,6 @@
       <c r="G121" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H121" s="2" t="inlineStr"/>
-      <c r="I121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr"/>
@@ -3793,8 +3530,6 @@
       <c r="G122" s="2" t="n">
         <v>116</v>
       </c>
-      <c r="H122" s="2" t="inlineStr"/>
-      <c r="I122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr"/>
@@ -3821,8 +3556,6 @@
       <c r="G123" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H123" s="2" t="inlineStr"/>
-      <c r="I123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr"/>
@@ -3852,8 +3585,6 @@
       <c r="G124" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H124" s="2" t="inlineStr"/>
-      <c r="I124" s="3" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr"/>
@@ -3880,8 +3611,6 @@
       <c r="G125" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="H125" s="2" t="inlineStr"/>
-      <c r="I125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr"/>
@@ -3908,8 +3637,6 @@
       <c r="G126" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H126" s="2" t="inlineStr"/>
-      <c r="I126" s="3" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr"/>
@@ -3933,8 +3660,6 @@
       <c r="G127" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H127" s="2" t="inlineStr"/>
-      <c r="I127" s="3" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr"/>
@@ -3970,8 +3695,6 @@
       <c r="G128" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H128" s="2" t="inlineStr"/>
-      <c r="I128" s="3" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr"/>
@@ -3995,8 +3718,6 @@
       <c r="G129" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H129" s="2" t="inlineStr"/>
-      <c r="I129" s="3" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr"/>
@@ -4022,8 +3743,6 @@
       <c r="G130" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H130" s="2" t="inlineStr"/>
-      <c r="I130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr"/>
@@ -4047,8 +3766,6 @@
       <c r="G131" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H131" s="2" t="inlineStr"/>
-      <c r="I131" s="3" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr"/>
@@ -4081,8 +3798,6 @@
       <c r="G132" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="H132" s="2" t="inlineStr"/>
-      <c r="I132" s="3" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr"/>
@@ -4106,8 +3821,6 @@
       <c r="G133" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H133" s="2" t="inlineStr"/>
-      <c r="I133" s="3" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr"/>
@@ -4135,8 +3848,6 @@
       <c r="G134" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H134" s="2" t="inlineStr"/>
-      <c r="I134" s="3" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr"/>
@@ -4160,8 +3871,6 @@
       <c r="G135" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H135" s="2" t="inlineStr"/>
-      <c r="I135" s="3" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr"/>
@@ -4185,8 +3894,6 @@
       <c r="G136" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H136" s="2" t="inlineStr"/>
-      <c r="I136" s="3" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr"/>
@@ -4210,1138 +3917,1387 @@
       <c r="G137" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H137" s="2" t="inlineStr"/>
-      <c r="I137" s="3" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" s="4" t="inlineStr">
+      <c r="A138" s="2" t="inlineStr">
         <is>
           <t>形式层（外观）</t>
         </is>
       </c>
-      <c r="B138" s="4" t="inlineStr">
+      <c r="B138" s="2" t="inlineStr">
         <is>
           <t>色彩、材质与饰面</t>
         </is>
       </c>
-      <c r="C138" s="4" t="inlineStr">
+      <c r="C138" s="2" t="inlineStr">
         <is>
           <t>色彩</t>
         </is>
       </c>
-      <c r="D138" s="4" t="inlineStr">
+      <c r="D138" s="2" t="inlineStr">
         <is>
           <t>色彩设计</t>
         </is>
       </c>
-      <c r="E138" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F138" s="5" t="inlineStr">
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="inlineStr">
+        <is>
+          <t>...nd sustainable produc- tion methods, is driving totally new colour design strategies and market- ing campaigns. 43 CMF DESIGN Several...</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr"/>
+      <c r="B139" s="2" t="inlineStr"/>
+      <c r="C139" s="2" t="inlineStr"/>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>配色方案</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
         <is>
           <t>...tinent and not influenced by a temporary fashion trend, the colour palettes have been applied to ma-terials and finishes including fab...</t>
         </is>
       </c>
-      <c r="G138" s="4" t="n">
+      <c r="G139" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr"/>
+      <c r="B140" s="2" t="inlineStr"/>
+      <c r="C140" s="2" t="inlineStr"/>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>色彩搭配</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F140" s="3" t="inlineStr">
+        <is>
+          <t>...ly used in younger consumer market segments. Since brighter colour combinations create a higher level of contrast, they also tend to becom...</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H138" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I138" s="5" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="4" t="inlineStr"/>
-      <c r="B139" s="4" t="inlineStr"/>
-      <c r="C139" s="4" t="inlineStr"/>
-      <c r="D139" s="4" t="inlineStr">
-        <is>
-          <t>配色方案</t>
-        </is>
-      </c>
-      <c r="E139" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F139" s="5" t="inlineStr">
-        <is>
-          <t>...tinent and not influenced by a temporary fashion trend, the colour palettes have been applied to ma-terials and finishes including fab...</t>
-        </is>
-      </c>
-      <c r="G139" s="4" t="n">
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr"/>
+      <c r="B141" s="2" t="inlineStr"/>
+      <c r="C141" s="2" t="inlineStr"/>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>色调</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>...Tech surface texture guidelines for plastic surfaces and Pantone books with colour chips for printing and paint. 59 CMF DESI...</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr"/>
+      <c r="B142" s="2" t="inlineStr"/>
+      <c r="C142" s="2" t="inlineStr"/>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>中性色</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="inlineStr">
+        <is>
+          <t>...ds but instead provide a longer and more durable aesthetic. Neutral tones are ideal for products intending to be in use for longer pe...</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr"/>
+      <c r="B143" s="2" t="inlineStr"/>
+      <c r="C143" s="2" t="inlineStr"/>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>色彩趋势</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>... D Oe conventions are independent of aesthetics or seasonal colour trends and tend to be very standardized across cultures and count...</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr"/>
+      <c r="B144" s="2" t="inlineStr"/>
+      <c r="C144" s="2" t="inlineStr"/>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>色彩心理学</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>...minate colour differences and tonality nuances. The lack of colour affinity is a common physiological condition known as colour blindne...</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H139" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I139" s="5" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="4" t="inlineStr"/>
-      <c r="B140" s="4" t="inlineStr"/>
-      <c r="C140" s="4" t="inlineStr"/>
-      <c r="D140" s="4" t="inlineStr">
-        <is>
-          <t>色彩搭配</t>
-        </is>
-      </c>
-      <c r="E140" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F140" s="5" t="inlineStr">
-        <is>
-          <t>...tegories have different market cycles, the same is true for colour combinations. Neutral tones (Quit) Neutral tones, including shades of g...</t>
-        </is>
-      </c>
-      <c r="G140" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H140" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I140" s="5" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="4" t="inlineStr"/>
-      <c r="B141" s="4" t="inlineStr"/>
-      <c r="C141" s="4" t="inlineStr"/>
-      <c r="D141" s="4" t="inlineStr">
-        <is>
-          <t>色调</t>
-        </is>
-      </c>
-      <c r="E141" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F141" s="5" t="inlineStr">
-        <is>
-          <t>...pplier. Existing standardized references systems include Pantone® and NCS® (Natural Colour System) for colours, Mold-Tech pl...</t>
-        </is>
-      </c>
-      <c r="G141" s="4" t="n">
-        <v>69</v>
-      </c>
-      <c r="H141" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I141" s="5" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="4" t="inlineStr"/>
-      <c r="B142" s="4" t="inlineStr"/>
-      <c r="C142" s="4" t="inlineStr"/>
-      <c r="D142" s="4" t="inlineStr">
-        <is>
-          <t>中性色</t>
-        </is>
-      </c>
-      <c r="E142" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F142" s="5" t="inlineStr">
-        <is>
-          <t>...d more classic look, which is also longer lasting. Although neutral tones are also influenced by trends, they don’t necessarily fall ...</t>
-        </is>
-      </c>
-      <c r="G142" s="4" t="n">
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr"/>
+      <c r="B145" s="2" t="inlineStr"/>
+      <c r="C145" s="2" t="inlineStr"/>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>色彩测量</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>...tor of the “glow in the dark” functionality. Wal CMF DESIGN COLOUR MEASURING TOOLS The process of colour matching is affected by many di...</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr"/>
+      <c r="B146" s="2" t="inlineStr"/>
+      <c r="C146" s="2" t="inlineStr"/>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>色彩语言</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>... Ray Eames. The Polaroid camera represents an iconic visual design language revolving around clear functional elements, highlighted by ...</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr"/>
+      <c r="B147" s="2" t="inlineStr"/>
+      <c r="C147" s="2" t="inlineStr"/>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>数字色彩</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>...sed business models have recently emerged, revolving around digital colour readers paired with the process of colour collecting, organ...</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr"/>
+      <c r="B148" s="2" t="inlineStr"/>
+      <c r="C148" s="2" t="inlineStr"/>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>色彩体系</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>... to the NCS Colourpin® and the scientific method of Natural Colour System, Nichetto Studio was able to extract a selection of colours...</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr"/>
+      <c r="B149" s="2" t="inlineStr"/>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>材质</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>材质</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>...elements are impossible to separate from one another. Every material has its own array of optimal manufacturing processes, which...</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="n">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr"/>
+      <c r="B150" s="2" t="inlineStr"/>
+      <c r="C150" s="2" t="inlineStr"/>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>材质设计</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>...rface development, serving a range of different industries. Material Design It generally consists of ideating new and connecting existi...</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr"/>
+      <c r="B151" s="2" t="inlineStr"/>
+      <c r="C151" s="2" t="inlineStr"/>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>触感</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>...lamb, goat and sometimes deer. Although suede has a natural soft touch surface, which is thin and pliable, it tends to be less dur...</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr"/>
+      <c r="B152" s="2" t="inlineStr"/>
+      <c r="C152" s="2" t="inlineStr"/>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>纹理</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>...DESIGN Acollection of different images, objects, materials, textures and key words, selected to create and communicate an engag...</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr"/>
+      <c r="B153" s="2" t="inlineStr"/>
+      <c r="C153" s="2" t="inlineStr"/>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>金属材质</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>...te visual characteristics of original precious minerals and metals in order to evoke a feeling of high end. Other materials h...</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr"/>
+      <c r="B154" s="2" t="inlineStr"/>
+      <c r="C154" s="2" t="inlineStr"/>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>铝合金</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>...ssicon. This lounge chair comprises a lightweight steel and aluminium framework with a stretched 3D woven textile mesh. The chair...</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr"/>
+      <c r="B155" s="2" t="inlineStr"/>
+      <c r="C155" s="2" t="inlineStr"/>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>不锈钢</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>...ar, corrosion and because of its anti-bacterial properties. Stainless steel is a very strong material that although it is hard to form,...</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H142" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I142" s="5" t="inlineStr"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="4" t="inlineStr"/>
-      <c r="B143" s="4" t="inlineStr"/>
-      <c r="C143" s="4" t="inlineStr"/>
-      <c r="D143" s="4" t="inlineStr">
-        <is>
-          <t>色彩趋势</t>
-        </is>
-      </c>
-      <c r="E143" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F143" s="5" t="inlineStr">
-        <is>
-          <t>... lathers. The books showcase the latest surface texture and colour trends with corresponding samples and inspiring visuals. 45 CMF D...</t>
-        </is>
-      </c>
-      <c r="G143" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H143" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I143" s="5" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="4" t="inlineStr"/>
-      <c r="B144" s="4" t="inlineStr"/>
-      <c r="C144" s="4" t="inlineStr"/>
-      <c r="D144" s="4" t="inlineStr">
-        <is>
-          <t>色彩心理学</t>
-        </is>
-      </c>
-      <c r="E144" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F144" s="5" t="inlineStr">
-        <is>
-          <t>...ssociated with cleanliness, decluttering and organizing. In colour psychology, it is known as a colour of fresh starts and new cre- ation...</t>
-        </is>
-      </c>
-      <c r="G144" s="4" t="n">
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr"/>
+      <c r="B156" s="2" t="inlineStr"/>
+      <c r="C156" s="2" t="inlineStr"/>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>碳纤维</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="inlineStr">
+        <is>
+          <t>...a modern upgrade with metal details and intaglio. Moreover, carbon fibre trim has a premium sport perception as it is used on compet...</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr"/>
+      <c r="B157" s="2" t="inlineStr"/>
+      <c r="C157" s="2" t="inlineStr"/>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>皮革</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>...or to the interior with many options for the various parts, leather seats, or even the stitching. apus tailor made- &gt;&gt; smart BR...</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr"/>
+      <c r="B158" s="2" t="inlineStr"/>
+      <c r="C158" s="2" t="inlineStr"/>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>木材</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>... moulded wooden-like surface texture. By moulding a natural wood grain into the plastic, an evocative visual and tactile ref...</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr"/>
+      <c r="B159" s="2" t="inlineStr"/>
+      <c r="C159" s="2" t="inlineStr"/>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>木饰面</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>...smoothen out surface imperfections. Consumer products using wood veneers, especially those expected to be in close contact with hum...</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr"/>
+      <c r="B160" s="2" t="inlineStr"/>
+      <c r="C160" s="2" t="inlineStr"/>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>玻璃</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F160" s="3" t="inlineStr">
+        <is>
+          <t>...ft touch for paint or plastic and anti-shatter coatings for glass. Different materials can withstand different levels of appl...</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr"/>
+      <c r="B161" s="2" t="inlineStr"/>
+      <c r="C161" s="2" t="inlineStr"/>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>塑料</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="inlineStr">
+        <is>
+          <t>... surface texture. By moulding a natural wood grain into the plastic, an evocative visual and tactile reference is created, maki...</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr"/>
+      <c r="B162" s="2" t="inlineStr"/>
+      <c r="C162" s="2" t="inlineStr"/>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>纺织品</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="inlineStr">
+        <is>
+          <t>...ed by manufacturing, where she became an expert in sourcing textiles, knits and communicating with vendors at Guess Apparel. Sh...</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr"/>
+      <c r="B163" s="2" t="inlineStr"/>
+      <c r="C163" s="2" t="inlineStr"/>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>天然材料</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>...rwise overly smooth and perfect glossy products. Wearing in Natural materials like wood, certain metals and leather, are expected to wea...</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr"/>
+      <c r="B164" s="2" t="inlineStr"/>
+      <c r="C164" s="2" t="inlineStr"/>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>合成材料</t>
+        </is>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>... abundant crops. It fixes nitrogen and reduces the need for synthetic fertilizers. Clovers occasionally have leaves with four lea...</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr"/>
+      <c r="B165" s="2" t="inlineStr"/>
+      <c r="C165" s="2" t="inlineStr"/>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>橡胶弹性体</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>...ough a co-moulding process. Once different materials — like rubber and plastic in this case — have been fused together, they b...</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr"/>
+      <c r="B166" s="2" t="inlineStr"/>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>表面处理</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>表面处理</t>
+        </is>
+      </c>
+      <c r="E166" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F166" s="3" t="inlineStr">
+        <is>
+          <t>...f coated with a glossy topcoat. A surface with a soft touch finish will make the colour slightly more muted and visually softe...</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="n">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr"/>
+      <c r="B167" s="2" t="inlineStr"/>
+      <c r="C167" s="2" t="inlineStr"/>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>表面装饰</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>...tals is recommended, as they are more likely to provide the surface decoration with a longer lifespan. PVD COATING PVD stands for Physical...</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H144" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I144" s="5" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="4" t="inlineStr"/>
-      <c r="B145" s="4" t="inlineStr"/>
-      <c r="C145" s="4" t="inlineStr"/>
-      <c r="D145" s="4" t="inlineStr">
-        <is>
-          <t>色彩测量</t>
-        </is>
-      </c>
-      <c r="E145" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F145" s="5" t="inlineStr">
-        <is>
-          <t>...tor of the “glow in the dark” functionality. Wal CMF DESIGN COLOUR MEASURING TOOLS The process of colour matching is affected by many di...</t>
-        </is>
-      </c>
-      <c r="G145" s="4" t="n">
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr"/>
+      <c r="B168" s="2" t="inlineStr"/>
+      <c r="C168" s="2" t="inlineStr"/>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>饰面</t>
+        </is>
+      </c>
+      <c r="E168" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F168" s="3" t="inlineStr">
+        <is>
+          <t>...statement. Some examples include novelty and unconventional surface finishes of high-end cars, which are either completely matte or co...</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr"/>
+      <c r="B169" s="2" t="inlineStr"/>
+      <c r="C169" s="2" t="inlineStr"/>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>抛光</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="inlineStr">
+        <is>
+          <t>...des being machined out of a single block of aluminium, were polished and finished by hand. The desk was produced by Neal Feay St...</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr"/>
+      <c r="B170" s="2" t="inlineStr"/>
+      <c r="C170" s="2" t="inlineStr"/>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>哑光</t>
+        </is>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F170" s="3" t="inlineStr">
+        <is>
+          <t>...e ultimate in premium for a car, and anything else for that matter. Plastic parts can be leather wrapped. Even the smallest a...</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr"/>
+      <c r="B171" s="2" t="inlineStr"/>
+      <c r="C171" s="2" t="inlineStr"/>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>光泽</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>...n, wood veneer, metal, etc.), the gloss level (satin, mate, glossy), the type of finish (brushed, sandblasted, polished for m...</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr"/>
+      <c r="B172" s="2" t="inlineStr"/>
+      <c r="C172" s="2" t="inlineStr"/>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>高光</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>... or the actual substrate material. Challenges 1. When using high gloss UV resistant topcoat, especially with a deep colour, the su...</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr"/>
+      <c r="B173" s="2" t="inlineStr"/>
+      <c r="C173" s="2" t="inlineStr"/>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>缎面</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>...lishing is used for mirror-like surfaces, sand-blasting for satin to matte surfaces and brushing for unidirectional satin sur...</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr"/>
+      <c r="B174" s="2" t="inlineStr"/>
+      <c r="C174" s="2" t="inlineStr"/>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>拉丝</t>
+        </is>
+      </c>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>...oducts, the polishing procedure is often performed by hand. Brushed aluminium is a very common trim used in several industries ...</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr"/>
+      <c r="B175" s="2" t="inlineStr"/>
+      <c r="C175" s="2" t="inlineStr"/>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>喷砂</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>...s level (satin, mate, glossy), the type of finish (brushed, sandblasted, polished for metal), and so on. CMF specs tend to be compl...</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H145" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I145" s="5" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="4" t="inlineStr"/>
-      <c r="B146" s="4" t="inlineStr"/>
-      <c r="C146" s="4" t="inlineStr"/>
-      <c r="D146" s="4" t="inlineStr">
-        <is>
-          <t>色彩语言</t>
-        </is>
-      </c>
-      <c r="E146" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F146" s="5" t="inlineStr">
-        <is>
-          <t>...because of its light weight. VISUAL DESIGN LANGUAGES Visual design languages are the overall composition of forms, lines, mate- rials a...</t>
-        </is>
-      </c>
-      <c r="G146" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="H146" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I146" s="5" t="inlineStr"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="4" t="inlineStr"/>
-      <c r="B147" s="4" t="inlineStr"/>
-      <c r="C147" s="4" t="inlineStr">
-        <is>
-          <t>材质</t>
-        </is>
-      </c>
-      <c r="D147" s="4" t="inlineStr">
-        <is>
-          <t>材质设计</t>
-        </is>
-      </c>
-      <c r="E147" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F147" s="5" t="inlineStr">
-        <is>
-          <t>...ributions. It is never recommended to decide on 2 colour or material combination without first visualizing it either digitally or physically...</t>
-        </is>
-      </c>
-      <c r="G147" s="4" t="n">
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr"/>
+      <c r="B176" s="2" t="inlineStr"/>
+      <c r="C176" s="2" t="inlineStr"/>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>激光加工</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>...roperly calibrated, burning marks can occur. 2. In general, laser markings or engravings on soft metals are likely to 162 METALS scra...</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr"/>
+      <c r="B177" s="2" t="inlineStr"/>
+      <c r="C177" s="2" t="inlineStr"/>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>涂层</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>...DESIGN Several companies, who are also suppliers of paints, coatings and pig- ments, create colour forecasting books and brochu...</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr"/>
+      <c r="B178" s="2" t="inlineStr"/>
+      <c r="C178" s="2" t="inlineStr"/>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>镀铬</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>...ial after used, so it is more environmentally friendly than chrome tanning. Challenges 1. When aniline tanning is used, the fi...</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr"/>
+      <c r="B179" s="2" t="inlineStr"/>
+      <c r="C179" s="2" t="inlineStr"/>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>涂料油漆</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="inlineStr">
+        <is>
+          <t>... core activities mostly happen in a lab, mixing of inks and paints in order to create nov- elty effects with strong technical...</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr"/>
+      <c r="B180" s="2" t="inlineStr"/>
+      <c r="C180" s="2" t="inlineStr"/>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>电化学蚀刻</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F180" s="3" t="inlineStr">
+        <is>
+          <t>...ture effect. There is also an etching process based on photochemical etching, which is utilized to produce high precision, flat metal pa...</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr"/>
+      <c r="B181" s="2" t="inlineStr"/>
+      <c r="C181" s="2" t="inlineStr"/>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>阳极化处理</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="inlineStr">
+        <is>
+          <t>...which can accept dyes easily. 161 CM F DESIGN Benefits ‘ 4. Anodised aluminium can be up to 50% more durable than alumin- jum on...</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr"/>
+      <c r="B182" s="2" t="inlineStr"/>
+      <c r="C182" s="2" t="inlineStr"/>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>模压成型</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>...cesses including co-moulding with rubber or silicone, rotor moulding and injection moulding. In terms of challenges, recycling c...</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr"/>
+      <c r="B183" s="2" t="inlineStr"/>
+      <c r="C183" s="2" t="inlineStr"/>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>注塑成型</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F183" s="3" t="inlineStr">
+        <is>
+          <t>... the touch. 168 PLASTICS MOST COMMON FINISHES AND PROCESSES INJECTION The process of plastic injection moulding is very common an...</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr"/>
+      <c r="B184" s="2" t="inlineStr"/>
+      <c r="C184" s="2" t="inlineStr"/>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>颜料</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F184" s="3" t="inlineStr">
+        <is>
+          <t>...g is affected by many different aspects such as the type of pigments utilized, the selected method of applica- tion and the bas...</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr"/>
+      <c r="B185" s="2" t="inlineStr"/>
+      <c r="C185" s="2" t="inlineStr"/>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>染料</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>...0 METALS The aluminium trays are hand-dipped in water-based dye, a process that resembles that of painting Easter eggs. Tra...</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr"/>
+      <c r="B186" s="2" t="inlineStr"/>
+      <c r="C186" s="2" t="inlineStr"/>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>金属闪光效果</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F186" s="3" t="inlineStr">
+        <is>
+          <t>...ond read will be the effect of the paint — glossy or matte, metallic flake or pearlescent effect, etc. Usually, the third read corresp...</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr"/>
+      <c r="B187" s="2" t="inlineStr"/>
+      <c r="C187" s="2" t="inlineStr"/>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>珠光效果</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="inlineStr">
+        <is>
+          <t>...fects applied through conventional spraying methods include pearlescent, metallic, magnetic patterns, colour shifting and soft touc...</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H147" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I147" s="5" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="4" t="inlineStr"/>
-      <c r="B148" s="4" t="inlineStr"/>
-      <c r="C148" s="4" t="inlineStr"/>
-      <c r="D148" s="4" t="inlineStr">
-        <is>
-          <t>触感</t>
-        </is>
-      </c>
-      <c r="E148" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F148" s="5" t="inlineStr">
-        <is>
-          <t>...f TPEs with more rigid materials provides prod- ucts with a soft touch feel while enhancing its ergonomics, strength and dimension...</t>
-        </is>
-      </c>
-      <c r="G148" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="H148" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I148" s="5" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="4" t="inlineStr"/>
-      <c r="B149" s="4" t="inlineStr"/>
-      <c r="C149" s="4" t="inlineStr"/>
-      <c r="D149" s="4" t="inlineStr">
-        <is>
-          <t>纹理</t>
-        </is>
-      </c>
-      <c r="E149" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F149" s="5" t="inlineStr">
-        <is>
-          <t>...created with an ultra-strong yard knit woven into different textures, shaping the form and eliminating unnecessary weight. Not ...</t>
-        </is>
-      </c>
-      <c r="G149" s="4" t="n">
-        <v>138</v>
-      </c>
-      <c r="H149" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I149" s="5" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="4" t="inlineStr"/>
-      <c r="B150" s="4" t="inlineStr"/>
-      <c r="C150" s="4" t="inlineStr"/>
-      <c r="D150" s="4" t="inlineStr">
-        <is>
-          <t>金属材质</t>
-        </is>
-      </c>
-      <c r="E150" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F150" s="5" t="inlineStr">
-        <is>
-          <t>...ources. Minerals like diamonds, crystal, glass and precious metals such as gold, platinum and titanium are at the top of the ...</t>
-        </is>
-      </c>
-      <c r="G150" s="4" t="n">
-        <v>172</v>
-      </c>
-      <c r="H150" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I150" s="5" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="4" t="inlineStr"/>
-      <c r="B151" s="4" t="inlineStr"/>
-      <c r="C151" s="4" t="inlineStr"/>
-      <c r="D151" s="4" t="inlineStr">
-        <is>
-          <t>铝合金</t>
-        </is>
-      </c>
-      <c r="E151" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F151" s="5" t="inlineStr">
-        <is>
-          <t>...ssembled allowing clear part separation between plastic and aluminium components. AA‘o34jqspe}O0 ee 0y9zqUesgud|u n} o\ovqo o y c...</t>
-        </is>
-      </c>
-      <c r="G151" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="H151" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I151" s="5" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="4" t="inlineStr"/>
-      <c r="B152" s="4" t="inlineStr"/>
-      <c r="C152" s="4" t="inlineStr"/>
-      <c r="D152" s="4" t="inlineStr">
-        <is>
-          <t>不锈钢</t>
-        </is>
-      </c>
-      <c r="E152" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F152" s="5" t="inlineStr">
-        <is>
-          <t>...ed at the same time. Within the medical field for instance, stainless steel is used in surgical tools because of its high resistance to...</t>
-        </is>
-      </c>
-      <c r="G152" s="4" t="n">
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr"/>
+      <c r="B188" s="2" t="inlineStr"/>
+      <c r="C188" s="2" t="inlineStr"/>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>缝线工艺</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F188" s="3" t="inlineStr">
+        <is>
+          <t>...y premium or luxury product categories as trim details (the stitching or piping for car seats) or as iconic branding ele- ments f...</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr"/>
+      <c r="B189" s="2" t="inlineStr"/>
+      <c r="C189" s="2" t="inlineStr"/>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>编织工艺</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F189" s="3" t="inlineStr">
+        <is>
+          <t>...e fact that the shoes are created with an ultra-strong yard knit woven into different textures, shaping the form and elimina...</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr"/>
+      <c r="B190" s="2" t="inlineStr"/>
+      <c r="C190" s="2" t="inlineStr"/>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>层压工艺</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F190" s="3" t="inlineStr">
+        <is>
+          <t>...pliances, car bumpers (PP), synthetic leather and synthetic laminates (PVC) and car interior and exterior parts and portable mobi...</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr"/>
+      <c r="B191" s="2" t="inlineStr"/>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>美学感知</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>奢华感</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>... countries perceive it as the colour of death and mourning. LUXURY STATUS ROYALTY NOBILITY CHURCH ROMANCE SPIRITUALITY IMAGINA...</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr"/>
+      <c r="B192" s="2" t="inlineStr"/>
+      <c r="C192" s="2" t="inlineStr"/>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>高端质感</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F192" s="3" t="inlineStr">
+        <is>
+          <t>...discard. In some cases though, bright tones are utilized by premium or luxury product categories as trim details (the stitching...</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr"/>
+      <c r="B193" s="2" t="inlineStr"/>
+      <c r="C193" s="2" t="inlineStr"/>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>情感化设计</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F193" s="3" t="inlineStr">
+        <is>
+          <t>...nd consumer segmentations; as it allows for the creation of emotional connections, added value and the fulfilment of certain huma...</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr"/>
+      <c r="B194" s="2" t="inlineStr"/>
+      <c r="C194" s="2" t="inlineStr"/>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>可持续设计</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="inlineStr">
+        <is>
+          <t>...nability POV, you are provided with materials that are 100% sustainable in the processes or, for instance in the case of leather, f...</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr"/>
+      <c r="B195" s="2" t="inlineStr"/>
+      <c r="C195" s="2" t="inlineStr"/>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>耐用性</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F195" s="3" t="inlineStr">
+        <is>
+          <t>...e and prestigious. As metals provide excellent rigidity and durability properties, they have the highest likelihood of all materia...</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="H152" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I152" s="5" t="inlineStr"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="4" t="inlineStr"/>
-      <c r="B153" s="4" t="inlineStr"/>
-      <c r="C153" s="4" t="inlineStr"/>
-      <c r="D153" s="4" t="inlineStr">
-        <is>
-          <t>碳纤维</t>
-        </is>
-      </c>
-      <c r="E153" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F153" s="5" t="inlineStr">
-        <is>
-          <t>...e touch — in order to guarantee the signature Detail of the carbon fibre structure of the BMW i3. 114 quality of the brand. This app...</t>
-        </is>
-      </c>
-      <c r="G153" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="H153" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I153" s="5" t="inlineStr"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="4" t="inlineStr"/>
-      <c r="B154" s="4" t="inlineStr"/>
-      <c r="C154" s="4" t="inlineStr"/>
-      <c r="D154" s="4" t="inlineStr">
-        <is>
-          <t>皮革</t>
-        </is>
-      </c>
-      <c r="E154" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F154" s="5" t="inlineStr">
-        <is>
-          <t>... with Nancy Holman 150 Metals 166 Plastics 174 Textiles 180 Leather 188 Wood 194 Glass 198 Coatings  Colour, Material and Finis...</t>
-        </is>
-      </c>
-      <c r="G154" s="4" t="n">
-        <v>135</v>
-      </c>
-      <c r="H154" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I154" s="5" t="inlineStr"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="4" t="inlineStr"/>
-      <c r="B155" s="4" t="inlineStr"/>
-      <c r="C155" s="4" t="inlineStr"/>
-      <c r="D155" s="4" t="inlineStr">
-        <is>
-          <t>木材</t>
-        </is>
-      </c>
-      <c r="E155" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F155" s="5" t="inlineStr">
-        <is>
-          <t>...d value spectrum. Transparent table by Nendo with a moulded wooden-like surface texture. By moulding a natural wood grain in...</t>
-        </is>
-      </c>
-      <c r="G155" s="4" t="n">
-        <v>91</v>
-      </c>
-      <c r="H155" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I155" s="5" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="4" t="inlineStr"/>
-      <c r="B156" s="4" t="inlineStr"/>
-      <c r="C156" s="4" t="inlineStr"/>
-      <c r="D156" s="4" t="inlineStr">
-        <is>
-          <t>玻璃</t>
-        </is>
-      </c>
-      <c r="E156" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F156" s="5" t="inlineStr">
-        <is>
-          <t>...o withstanding dents and scratches. Rigid materials such as glass or brittle plastics on the other hand, are more prone to br...</t>
-        </is>
-      </c>
-      <c r="G156" s="4" t="n">
-        <v>63</v>
-      </c>
-      <c r="H156" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I156" s="5" t="inlineStr"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="4" t="inlineStr"/>
-      <c r="B157" s="4" t="inlineStr"/>
-      <c r="C157" s="4" t="inlineStr"/>
-      <c r="D157" s="4" t="inlineStr">
-        <is>
-          <t>塑料</t>
-        </is>
-      </c>
-      <c r="E157" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F157" s="5" t="inlineStr">
-        <is>
-          <t>...issues. Another aspect that aids the low perceived value of plastic is its ease of manufacturing which allows for the productio...</t>
-        </is>
-      </c>
-      <c r="G157" s="4" t="n">
-        <v>133</v>
-      </c>
-      <c r="H157" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I157" s="5" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="4" t="inlineStr"/>
-      <c r="B158" s="4" t="inlineStr"/>
-      <c r="C158" s="4" t="inlineStr"/>
-      <c r="D158" s="4" t="inlineStr">
-        <is>
-          <t>纺织品</t>
-        </is>
-      </c>
-      <c r="E158" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F158" s="5" t="inlineStr">
-        <is>
-          <t>...de a broad range of natural and synthetic laminates, paper, textiles, carpets and upholstery utilized for home furnishings, app...</t>
-        </is>
-      </c>
-      <c r="G158" s="4" t="n">
-        <v>127</v>
-      </c>
-      <c r="H158" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I158" s="5" t="inlineStr"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="4" t="inlineStr"/>
-      <c r="B159" s="4" t="inlineStr"/>
-      <c r="C159" s="4" t="inlineStr">
-        <is>
-          <t>表面处理</t>
-        </is>
-      </c>
-      <c r="D159" s="4" t="inlineStr">
-        <is>
-          <t>表面处理</t>
-        </is>
-      </c>
-      <c r="E159" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F159" s="5" t="inlineStr">
-        <is>
-          <t>...ty of the material, the right types of dies, and its unique finishing processes. The hand and colour of a leather piece dyed w...</t>
-        </is>
-      </c>
-      <c r="G159" s="4" t="n">
-        <v>318</v>
-      </c>
-      <c r="H159" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I159" s="5" t="inlineStr"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="4" t="inlineStr"/>
-      <c r="B160" s="4" t="inlineStr"/>
-      <c r="C160" s="4" t="inlineStr"/>
-      <c r="D160" s="4" t="inlineStr">
-        <is>
-          <t>饰面</t>
-        </is>
-      </c>
-      <c r="E160" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F160" s="5" t="inlineStr">
-        <is>
-          <t>...d. This can be achieved through the use of low-cost novelty surface finishes, eye-catching colour combinations, or by creating an over...</t>
-        </is>
-      </c>
-      <c r="G160" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="H160" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I160" s="5" t="inlineStr"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="4" t="inlineStr"/>
-      <c r="B161" s="4" t="inlineStr"/>
-      <c r="C161" s="4" t="inlineStr"/>
-      <c r="D161" s="4" t="inlineStr">
-        <is>
-          <t>抛光</t>
-        </is>
-      </c>
-      <c r="E161" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F161" s="5" t="inlineStr">
-        <is>
-          <t>...tones. Moreover, if the dark surface has a glossy or highly polished finish, it will reveal oil marks from fingerprints, unless ...</t>
-        </is>
-      </c>
-      <c r="G161" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H161" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I161" s="5" t="inlineStr"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="4" t="inlineStr"/>
-      <c r="B162" s="4" t="inlineStr"/>
-      <c r="C162" s="4" t="inlineStr"/>
-      <c r="D162" s="4" t="inlineStr">
-        <is>
-          <t>哑光</t>
-        </is>
-      </c>
-      <c r="E162" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F162" s="5" t="inlineStr">
-        <is>
-          <t>...the second read will be the effect of the paint — glossy or matte, metallic flake or pearlescent effect, etc. Usually, the th...</t>
-        </is>
-      </c>
-      <c r="G162" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="H162" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I162" s="5" t="inlineStr"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="4" t="inlineStr"/>
-      <c r="B163" s="4" t="inlineStr"/>
-      <c r="C163" s="4" t="inlineStr"/>
-      <c r="D163" s="4" t="inlineStr">
-        <is>
-          <t>光泽</t>
-        </is>
-      </c>
-      <c r="E163" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F163" s="5" t="inlineStr">
-        <is>
-          <t>...the type of material (resin, wood veneer, metal, etc.), the gloss level (satin, mate, glossy), the type of finish (brushed, s...</t>
-        </is>
-      </c>
-      <c r="G163" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="H163" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I163" s="5" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="4" t="inlineStr"/>
-      <c r="B164" s="4" t="inlineStr"/>
-      <c r="C164" s="4" t="inlineStr"/>
-      <c r="D164" s="4" t="inlineStr">
-        <is>
-          <t>拉丝</t>
-        </is>
-      </c>
-      <c r="E164" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F164" s="5" t="inlineStr">
-        <is>
-          <t>...o the frame trim — the visible parts need to be polished or brushed by hand afterwards in order to create a pleasant surface fi...</t>
-        </is>
-      </c>
-      <c r="G164" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="H164" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I164" s="5" t="inlineStr"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="4" t="inlineStr"/>
-      <c r="B165" s="4" t="inlineStr"/>
-      <c r="C165" s="4" t="inlineStr"/>
-      <c r="D165" s="4" t="inlineStr">
-        <is>
-          <t>喷砂</t>
-        </is>
-      </c>
-      <c r="E165" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F165" s="5" t="inlineStr">
-        <is>
-          <t>...s level (satin, mate, glossy), the type of finish (brushed, sandblasted, polished for metal), and so on. CMF specs tend to be compl...</t>
-        </is>
-      </c>
-      <c r="G165" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H165" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I165" s="5" t="inlineStr"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="4" t="inlineStr"/>
-      <c r="B166" s="4" t="inlineStr"/>
-      <c r="C166" s="4" t="inlineStr"/>
-      <c r="D166" s="4" t="inlineStr">
-        <is>
-          <t>激光加工</t>
-        </is>
-      </c>
-      <c r="E166" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F166" s="5" t="inlineStr">
-        <is>
-          <t>...cutting in order to obtain a level of maximum precision. 2. Laser marking is a chemical and residue-free process, which can last long...</t>
-        </is>
-      </c>
-      <c r="G166" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="H166" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I166" s="5" t="inlineStr"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="4" t="inlineStr"/>
-      <c r="B167" s="4" t="inlineStr"/>
-      <c r="C167" s="4" t="inlineStr"/>
-      <c r="D167" s="4" t="inlineStr">
-        <is>
-          <t>涂层</t>
-        </is>
-      </c>
-      <c r="E167" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F167" s="5" t="inlineStr">
-        <is>
-          <t>...f the work in this area is currently directed to paints and coatings development for automotive interiors and exteriors, or for...</t>
-        </is>
-      </c>
-      <c r="G167" s="4" t="n">
-        <v>157</v>
-      </c>
-      <c r="H167" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I167" s="5" t="inlineStr"/>
-    </row>
-    <row r="168">
-      <c r="A168" s="4" t="inlineStr"/>
-      <c r="B168" s="4" t="inlineStr"/>
-      <c r="C168" s="4" t="inlineStr"/>
-      <c r="D168" s="4" t="inlineStr">
-        <is>
-          <t>镀铬</t>
-        </is>
-      </c>
-      <c r="E168" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F168" s="5" t="inlineStr">
-        <is>
-          <t>...osed to split or bonded leather. 183 CMF DESIGN Benefits 1. Chrome tanning is a quick process that provides the leather pieces...</t>
-        </is>
-      </c>
-      <c r="G168" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H168" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I168" s="5" t="inlineStr"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="4" t="inlineStr"/>
-      <c r="B169" s="4" t="inlineStr"/>
-      <c r="C169" s="4" t="inlineStr"/>
-      <c r="D169" s="4" t="inlineStr">
-        <is>
-          <t>油漆</t>
-        </is>
-      </c>
-      <c r="E169" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F169" s="5" t="inlineStr">
-        <is>
-          <t>...pment This area involves professional exterior and interior paint and finish developers, who have a strong chemistry backgrou...</t>
-        </is>
-      </c>
-      <c r="G169" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="H169" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I169" s="5" t="inlineStr"/>
-    </row>
-    <row r="170">
-      <c r="A170" s="4" t="inlineStr"/>
-      <c r="B170" s="4" t="inlineStr"/>
-      <c r="C170" s="4" t="inlineStr"/>
-      <c r="D170" s="4" t="inlineStr">
-        <is>
-          <t>电化学蚀刻</t>
-        </is>
-      </c>
-      <c r="E170" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F170" s="5" t="inlineStr">
-        <is>
-          <t>...dustries including aerospace and medical. The decoration in chemical etching is done by applying a layer of a selective coating, which w...</t>
-        </is>
-      </c>
-      <c r="G170" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="H170" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I170" s="5" t="inlineStr"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="4" t="inlineStr"/>
-      <c r="B171" s="4" t="inlineStr"/>
-      <c r="C171" s="4" t="inlineStr">
-        <is>
-          <t>美学感知</t>
-        </is>
-      </c>
-      <c r="D171" s="4" t="inlineStr">
-        <is>
-          <t>感知价值</t>
-        </is>
-      </c>
-      <c r="E171" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F171" s="5" t="inlineStr">
-        <is>
-          <t>..., higher perfor- mance and therefore, a higher price point. Perceived value on the other hand, can be created in order to provide a pro...</t>
-        </is>
-      </c>
-      <c r="G171" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="H171" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I171" s="5" t="inlineStr">
-        <is>
-          <t>（与“战略层&gt;意义创新&gt;情感与体验&gt;感知价值”为同一中文词，主归属该维度；此处为CMF专著补充的次归属，标注交叉引用，不重复计数）</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="4" t="inlineStr"/>
-      <c r="B172" s="4" t="inlineStr"/>
-      <c r="C172" s="4" t="inlineStr"/>
-      <c r="D172" s="4" t="inlineStr">
-        <is>
-          <t>奢华感</t>
-        </is>
-      </c>
-      <c r="E172" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F172" s="5" t="inlineStr">
-        <is>
-          <t>...ry to royalty and the nobility make purple also a colour of luxury and wealth with regal, extravagant qualities to it. Western...</t>
-        </is>
-      </c>
-      <c r="G172" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="H172" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I172" s="5" t="inlineStr"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="4" t="inlineStr"/>
-      <c r="B173" s="4" t="inlineStr"/>
-      <c r="C173" s="4" t="inlineStr"/>
-      <c r="D173" s="4" t="inlineStr">
-        <is>
-          <t>高端质感</t>
-        </is>
-      </c>
-      <c r="E173" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F173" s="5" t="inlineStr">
-        <is>
-          <t>...as textures, trims and other visual effects. In the case of premium products, elements such as tone on tone stitching or tone o...</t>
-        </is>
-      </c>
-      <c r="G173" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="H173" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I173" s="5" t="inlineStr"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="4" t="inlineStr"/>
-      <c r="B174" s="4" t="inlineStr"/>
-      <c r="C174" s="4" t="inlineStr"/>
-      <c r="D174" s="4" t="inlineStr">
-        <is>
-          <t>情感化设计</t>
-        </is>
-      </c>
-      <c r="E174" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F174" s="5" t="inlineStr">
-        <is>
-          <t>...n granted by the CMF design approach, triggers an immediate emotional connection. Besides the practical and the more intuitive kn...</t>
-        </is>
-      </c>
-      <c r="G174" s="4" t="n">
-        <v>67</v>
-      </c>
-      <c r="H174" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I174" s="5" t="inlineStr"/>
-    </row>
-    <row r="175">
-      <c r="A175" s="4" t="inlineStr"/>
-      <c r="B175" s="4" t="inlineStr"/>
-      <c r="C175" s="4" t="inlineStr"/>
-      <c r="D175" s="4" t="inlineStr">
-        <is>
-          <t>可持续设计</t>
-        </is>
-      </c>
-      <c r="E175" s="5" t="inlineStr">
-        <is>
-          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra，2016）</t>
-        </is>
-      </c>
-      <c r="F175" s="5" t="inlineStr">
-        <is>
-          <t>...g behind the brand message that makes it validated within a sustainable point of view. Have you provided a compelling product for y...</t>
-        </is>
-      </c>
-      <c r="G175" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H175" s="4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I175" s="5" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr"/>
+      <c r="B196" s="2" t="inlineStr"/>
+      <c r="C196" s="2" t="inlineStr"/>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>工艺美感</t>
+        </is>
+      </c>
+      <c r="E196" s="3" t="inlineStr">
+        <is>
+          <t>《The Fundamental Principles of CMF Colour, Material and Finish Design》（Liliana Becerra, 2016，英文专著）</t>
+        </is>
+      </c>
+      <c r="F196" s="3" t="inlineStr">
+        <is>
+          <t>...ity. In addition, natural wood imparts a sense of class and craftsmanship. Recently, wood has received a modern upgrade with metal de...</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>